<commit_message>
STRAT05 and STRAT10 modifications
</commit_message>
<xml_diff>
--- a/lottery_config.xlsx
+++ b/lottery_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV_AREA\lottery_predictor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D6216C1-07A5-4A03-A2FE-7C5400894EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4706F3-0956-4399-A237-27AAA8454280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1365" yWindow="330" windowWidth="22800" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>lottery_name</t>
   </si>
@@ -159,13 +159,16 @@
   </si>
   <si>
     <t>Number of recent windows to use for confidence calculation</t>
+  </si>
+  <si>
+    <t>max_draws_to_use</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -184,6 +187,18 @@
       <sz val="9"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -212,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -226,6 +241,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,7 +583,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -709,7 +734,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" customWidth="1"/>
@@ -729,57 +754,66 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="4">
-        <v>100</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
+      <c r="A2" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="7">
+        <v>1000</v>
+      </c>
+      <c r="C2" s="6"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B3" s="4">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B4" s="4">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B5" s="4">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="4">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B7" s="4">
         <v>3</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>